<commit_message>
Various Awakeners Translated and Voiceline.
</commit_message>
<xml_diff>
--- a/TRANSLATIONS/01_UPLOAD_YOUR_CONTRIBUTIONS/vi/VN_Contributions_Ani0627.xlsx
+++ b/TRANSLATIONS/01_UPLOAD_YOUR_CONTRIBUTIONS/vi/VN_Contributions_Ani0627.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\MRMS TRANS\Source\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\MRMS TRANS\Source\0627 Work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{22C81D6F-4828-4A4F-BF3D-5012D70E706A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA26FE0C-8C6E-40E1-AEB4-C8336DDF1AE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32040" yWindow="1305" windowWidth="21600" windowHeight="11295" xr2:uid="{C33A330E-AEC1-4C37-91BA-26A733997407}"/>
+    <workbookView xWindow="34830" yWindow="795" windowWidth="21600" windowHeight="11295" xr2:uid="{C33A330E-AEC1-4C37-91BA-26A733997407}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="325">
   <si>
     <t>LanguageConfig_OverLimitUtlSkill_CN</t>
   </si>
@@ -1012,6 +1012,18 @@
   </si>
   <si>
     <t>bzvy</t>
+  </si>
+  <si>
+    <t>AwakerPotency_13303_PotencyName</t>
+  </si>
+  <si>
+    <t>asXv</t>
+  </si>
+  <si>
+    <t>花与诗的重逢</t>
+  </si>
+  <si>
+    <t>Cành Hoa Con Chữ \nTương Phùng Từ Duyên</t>
   </si>
 </sst>
 </file>
@@ -1393,7 +1405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50903D1D-E645-4DA5-AA35-41B4DF873A32}">
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -3910,6 +3922,35 @@
         <v>316</v>
       </c>
     </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>321</v>
+      </c>
+      <c r="B89" t="s">
+        <v>322</v>
+      </c>
+      <c r="C89" t="s">
+        <v>16</v>
+      </c>
+      <c r="D89">
+        <v>115</v>
+      </c>
+      <c r="E89" t="s">
+        <v>17</v>
+      </c>
+      <c r="F89" t="s">
+        <v>18</v>
+      </c>
+      <c r="G89" t="s">
+        <v>284</v>
+      </c>
+      <c r="H89" t="s">
+        <v>323</v>
+      </c>
+      <c r="I89" t="s">
+        <v>324</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>